<commit_message>
Expand East Asia search coverage
</commit_message>
<xml_diff>
--- a/outputs/phd_msc_opportunity_tracker.xlsx
+++ b/outputs/phd_msc_opportunity_tracker.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R64c327b5a64f45a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="2" r:id="R4f168ad93ee34ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Bank" sheetId="3" r:id="R9b621054aa234f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Source Plan" sheetId="4" r:id="R3eac23a05bb74876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual LinkedIn Capture" sheetId="5" r:id="R5b1e76fbb06a41b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Templates" sheetId="6" r:id="Rab903723e7964c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="7" r:id="R582cf78bd26a455c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" r:id="Rdb5acf9f61d34b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R120fb589bb3a4d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="2" r:id="R785f725d092b44dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Bank" sheetId="3" r:id="R0b5e5f6a7ccf47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Source Plan" sheetId="4" r:id="Rd913cb5f6d7b4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual LinkedIn Capture" sheetId="5" r:id="Re79f567b51db4baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Templates" sheetId="6" r:id="Rca33c9df93634c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="7" r:id="R4a7a56592f0c4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" r:id="Ra8744eddab824297"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -237,7 +237,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Alimi Muhammad Adewale" id="{8E6AA6AF-B31E-4128-8107-8EAEC75A20DE}"/>
+  <xltc:person displayName="Alimi Muhammad Adewale" id="{E8374112-964F-4DCC-882F-6E1CD3A4BD3E}"/>
 </xltc:personList>
 </file>
 
@@ -277,7 +277,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="LinkedInSearchesTable" displayName="LinkedInSearchesTable" ref="A4:F24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="LinkedInSearchesTable" displayName="LinkedInSearchesTable" ref="A4:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Search Name"/>
@@ -291,7 +291,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PublicSearchesTable" displayName="PublicSearchesTable" ref="A4:F38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PublicSearchesTable" displayName="PublicSearchesTable" ref="A4:F78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Cadence"/>
     <x:tableColumn id="2" name="Search Query"/>
@@ -4518,7 +4518,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56fc0029391846be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80873b88b0b844ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4826,10 +4826,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
-        <x:v>("University of Oxford") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery")</x:v>
+        <x:v>("University of Oxford") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Oxford%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Oxford%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F17" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4846,10 +4846,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D18" s="26" t="str">
-        <x:v>("University of Oxford") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil")</x:v>
+        <x:v>("University of Oxford") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
       </x:c>
       <x:c r="E18" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Oxford%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Oxford%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F18" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4866,10 +4866,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D19" s="26" t="str">
-        <x:v>("University of Cambridge") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery")</x:v>
+        <x:v>("University of Cambridge") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
       </x:c>
       <x:c r="E19" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Cambridge%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Cambridge%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F19" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4886,10 +4886,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D20" s="26" t="str">
-        <x:v>("University of Cambridge") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil")</x:v>
+        <x:v>("University of Cambridge") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
       </x:c>
       <x:c r="E20" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Cambridge%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Cambridge%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F20" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4906,10 +4906,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D21" s="26" t="str">
-        <x:v>("University of Toronto") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery")</x:v>
+        <x:v>("University of Toronto") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
       </x:c>
       <x:c r="E21" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Toronto%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Toronto%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F21" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4926,10 +4926,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D22" s="26" t="str">
-        <x:v>("University of Toronto") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil")</x:v>
+        <x:v>("University of Toronto") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
       </x:c>
       <x:c r="E22" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Toronto%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Toronto%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F22" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4946,10 +4946,10 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D23" s="26" t="str">
-        <x:v>("University of Michigan") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery")</x:v>
+        <x:v>("University of Michigan") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
       </x:c>
       <x:c r="E23" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Michigan%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Michigan%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F23" s="26" t="str">
         <x:v>Manual search only</x:v>
@@ -4966,12 +4966,812 @@
         <x:v>Twice weekly</x:v>
       </x:c>
       <x:c r="D24" s="26" t="str">
-        <x:v>("University of Michigan") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil")</x:v>
+        <x:v>("University of Michigan") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
       </x:c>
       <x:c r="E24" s="26" t="str">
-        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Michigan%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Michigan%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
       </x:c>
       <x:c r="F24" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Seoul National University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>("Seoul National University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Seoul%20National%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="str">
+        <x:v>Seoul National University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>("Seoul National University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Seoul%20National%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B27" s="26" t="str">
+        <x:v>KAIST - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C27" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D27" s="26" t="str">
+        <x:v>("KAIST") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E27" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22KAIST%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F27" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B28" s="26" t="str">
+        <x:v>KAIST - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C28" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D28" s="26" t="str">
+        <x:v>("KAIST") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E28" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22KAIST%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F28" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B29" s="26" t="str">
+        <x:v>Yonsei University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C29" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D29" s="26" t="str">
+        <x:v>("Yonsei University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E29" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Yonsei%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F29" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B30" s="26" t="str">
+        <x:v>Yonsei University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C30" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D30" s="26" t="str">
+        <x:v>("Yonsei University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E30" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Yonsei%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F30" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B31" s="26" t="str">
+        <x:v>Korea University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C31" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D31" s="26" t="str">
+        <x:v>("Korea University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E31" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Korea%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F31" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B32" s="26" t="str">
+        <x:v>Korea University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C32" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D32" s="26" t="str">
+        <x:v>("Korea University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E32" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Korea%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F32" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B33" s="26" t="str">
+        <x:v>POSTECH - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C33" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D33" s="26" t="str">
+        <x:v>("POSTECH") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E33" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22POSTECH%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F33" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B34" s="26" t="str">
+        <x:v>POSTECH - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C34" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D34" s="26" t="str">
+        <x:v>("POSTECH") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E34" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22POSTECH%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F34" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B35" s="26" t="str">
+        <x:v>Sungkyunkwan University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C35" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D35" s="26" t="str">
+        <x:v>("Sungkyunkwan University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E35" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Sungkyunkwan%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F35" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B36" s="26" t="str">
+        <x:v>Sungkyunkwan University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C36" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D36" s="26" t="str">
+        <x:v>("Sungkyunkwan University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E36" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Sungkyunkwan%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F36" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B37" s="26" t="str">
+        <x:v>Hanyang University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C37" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D37" s="26" t="str">
+        <x:v>("Hanyang University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E37" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Hanyang%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F37" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B38" s="26" t="str">
+        <x:v>Hanyang University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C38" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D38" s="26" t="str">
+        <x:v>("Hanyang University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E38" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Hanyang%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F38" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B39" s="26" t="str">
+        <x:v>Ulsan National Institute of Science and Technology - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C39" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D39" s="26" t="str">
+        <x:v>("Ulsan National Institute of Science and Technology") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E39" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Ulsan%20National%20Institute%20of%20Science%20and%20Technology%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F39" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>Ulsan National Institute of Science and Technology - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>("Ulsan National Institute of Science and Technology") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Ulsan%20National%20Institute%20of%20Science%20and%20Technology%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F40" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B41" s="26" t="str">
+        <x:v>GIST - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C41" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="str">
+        <x:v>("GIST") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E41" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22GIST%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F41" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B42" s="26" t="str">
+        <x:v>GIST - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C42" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D42" s="26" t="str">
+        <x:v>("GIST") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E42" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22GIST%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F42" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B43" s="26" t="str">
+        <x:v>Kyung Hee University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C43" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D43" s="26" t="str">
+        <x:v>("Kyung Hee University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E43" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyung%20Hee%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F43" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B44" s="26" t="str">
+        <x:v>Kyung Hee University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C44" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D44" s="26" t="str">
+        <x:v>("Kyung Hee University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E44" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyung%20Hee%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F44" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B45" s="26" t="str">
+        <x:v>University of Tokyo - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C45" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D45" s="26" t="str">
+        <x:v>("University of Tokyo") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E45" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Tokyo%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F45" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B46" s="26" t="str">
+        <x:v>University of Tokyo - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>("University of Tokyo") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Tokyo%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F46" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B47" s="26" t="str">
+        <x:v>Kyoto University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C47" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>("Kyoto University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyoto%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F47" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="str">
+        <x:v>Kyoto University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C48" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>("Kyoto University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyoto%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F48" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B49" s="26" t="str">
+        <x:v>Osaka University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C49" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>("Osaka University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Osaka%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F49" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B50" s="26" t="str">
+        <x:v>Osaka University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C50" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>("Osaka University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Osaka%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F50" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B51" s="26" t="str">
+        <x:v>Tohoku University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C51" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>("Tohoku University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Tohoku%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F51" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B52" s="26" t="str">
+        <x:v>Tohoku University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C52" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>("Tohoku University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Tohoku%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F52" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B53" s="26" t="str">
+        <x:v>Nagoya University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C53" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>("Nagoya University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Nagoya%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F53" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B54" s="26" t="str">
+        <x:v>Nagoya University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C54" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>("Nagoya University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Nagoya%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F54" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B55" s="26" t="str">
+        <x:v>Kyushu University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C55" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>("Kyushu University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyushu%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F55" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B56" s="26" t="str">
+        <x:v>Kyushu University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C56" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D56" s="26" t="str">
+        <x:v>("Kyushu University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Kyushu%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F56" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B57" s="26" t="str">
+        <x:v>Hokkaido University - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C57" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D57" s="26" t="str">
+        <x:v>("Hokkaido University") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Hokkaido%20University%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F57" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B58" s="26" t="str">
+        <x:v>Hokkaido University - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C58" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D58" s="26" t="str">
+        <x:v>("Hokkaido University") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Hokkaido%20University%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F58" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B59" s="26" t="str">
+        <x:v>University of Tsukuba - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C59" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>("University of Tsukuba") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Tsukuba%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B60" s="26" t="str">
+        <x:v>University of Tsukuba - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C60" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D60" s="26" t="str">
+        <x:v>("University of Tsukuba") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E60" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22University%20of%20Tsukuba%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F60" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B61" s="26" t="str">
+        <x:v>Institute of Science Tokyo - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C61" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D61" s="26" t="str">
+        <x:v>("Institute of Science Tokyo") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E61" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Institute%20of%20Science%20Tokyo%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F61" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B62" s="26" t="str">
+        <x:v>Institute of Science Tokyo - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C62" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D62" s="26" t="str">
+        <x:v>("Institute of Science Tokyo") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E62" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Institute%20of%20Science%20Tokyo%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F62" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B63" s="26" t="str">
+        <x:v>Okinawa Institute of Science and Technology - Drug Discovery</x:v>
+      </x:c>
+      <x:c r="C63" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D63" s="26" t="str">
+        <x:v>("Okinawa Institute of Science and Technology") AND ("PhD position" OR "DPhil" OR "PhD studentship" OR "doctoral" OR "graduate student") AND ("medicinal chemistry" OR "computational chemistry" OR "chemical biology" OR "drug discovery" OR "pharmaceutical sciences")</x:v>
+      </x:c>
+      <x:c r="E63" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Okinawa%20Institute%20of%20Science%20and%20Technology%22)%20AND%20(%22PhD%20position%22%20OR%20%22DPhil%22%20OR%20%22PhD%20studentship%22%20OR%20%22doctoral%22%20OR%20%22graduate%20student%22)%20AND%20(%22medicinal%20chemistry%22%20OR%20%22computational%20chemistry%22%20OR%20%22chemical%20biology%22%20OR%20%22drug%20discovery%22%20OR%20%22pharmaceutical%20sciences%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F63" s="26" t="str">
+        <x:v>Manual search only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="26" t="str">
+        <x:v>Posts</x:v>
+      </x:c>
+      <x:c r="B64" s="26" t="str">
+        <x:v>Okinawa Institute of Science and Technology - Health Informatics</x:v>
+      </x:c>
+      <x:c r="C64" s="26" t="str">
+        <x:v>Twice weekly</x:v>
+      </x:c>
+      <x:c r="D64" s="26" t="str">
+        <x:v>("Okinawa Institute of Science and Technology") AND ("health informatics" OR "digital health" OR "AI for health" OR "health data" OR "medical AI" OR "biomedical informatics") AND ("PhD" OR "DPhil" OR "MSc" OR "MPhil" OR "doctoral")</x:v>
+      </x:c>
+      <x:c r="E64" s="26" t="str">
+        <x:v>https://www.linkedin.com/search/results/content/?keywords=(%22Okinawa%20Institute%20of%20Science%20and%20Technology%22)%20AND%20(%22health%20informatics%22%20OR%20%22digital%20health%22%20OR%20%22AI%20for%20health%22%20OR%20%22health%20data%22%20OR%20%22medical%20AI%22%20OR%20%22biomedical%20informatics%22)%20AND%20(%22PhD%22%20OR%20%22DPhil%22%20OR%20%22MSc%22%20OR%20%22MPhil%22%20OR%20%22doctoral%22)&amp;origin=GLOBAL_SEARCH_HEADER</x:v>
+      </x:c>
+      <x:c r="F64" s="26" t="str">
         <x:v>Manual search only</x:v>
       </x:c>
     </x:row>
@@ -4982,7 +5782,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R606ef2d047ab48d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re08faf6085294ada"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5850,7 @@
         <x:v>https://www.google.com/search?q=%22PhD%20position%22%20%22medicinal%20chemistry%22%20%22fully%20funded%22</x:v>
       </x:c>
       <x:c r="D5" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E5" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5070,7 +5870,7 @@
         <x:v>https://www.google.com/search?q=%22PhD%20studentship%22%20%22drug%20discovery%22%20%22international%20students%22</x:v>
       </x:c>
       <x:c r="D6" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E6" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5090,7 +5890,7 @@
         <x:v>https://www.google.com/search?q=%22computational%20drug%20discovery%22%20%22PhD%20position%22</x:v>
       </x:c>
       <x:c r="D7" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E7" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5110,7 +5910,7 @@
         <x:v>https://www.google.com/search?q=%22health%20informatics%22%20%22PhD%22%20%22fully%20funded%22</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5130,7 +5930,7 @@
         <x:v>https://www.google.com/search?q=%22digital%20health%22%20%22PhD%20studentship%22</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E9" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5150,7 +5950,7 @@
         <x:v>https://www.google.com/search?q=%22AI%20for%20health%22%20%22PhD%20position%22%20%22health%20data%22</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5170,7 +5970,7 @@
         <x:v>https://www.google.com/search?q=%22natural%20product%20chemistry%22%20%22PhD%20position%22</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5190,7 +5990,7 @@
         <x:v>https://www.google.com/search?q=%22leishmaniasis%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5210,7 +6010,7 @@
         <x:v>https://www.google.com/search?q=%22molecular%20docking%22%20%22ADMET%22%20%22PhD%20position%22</x:v>
       </x:c>
       <x:c r="D13" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E13" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5230,7 +6030,7 @@
         <x:v>https://www.google.com/search?q=%22pharmaceutical%20supply%20chain%22%20%22PhD%22%20%22health%20systems%22</x:v>
       </x:c>
       <x:c r="D14" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5250,7 +6050,7 @@
         <x:v>https://www.google.com/search?q=%22University%20of%20Oxford%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5270,7 +6070,7 @@
         <x:v>https://www.google.com/search?q=%22University%20of%20Cambridge%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5290,7 +6090,7 @@
         <x:v>https://www.google.com/search?q=%22University%20of%20Toronto%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D17" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E17" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5310,7 +6110,7 @@
         <x:v>https://www.google.com/search?q=%22University%20of%20Michigan%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D18" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E18" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5330,7 +6130,7 @@
         <x:v>https://www.google.com/search?q=%22Nantes%20Universite%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D19" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E19" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5350,7 +6150,7 @@
         <x:v>https://www.google.com/search?q=%22McGill%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D20" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E20" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5370,7 +6170,7 @@
         <x:v>https://www.google.com/search?q=%22University%20of%20British%20Columbia%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D21" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E21" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5390,7 +6190,7 @@
         <x:v>https://www.google.com/search?q=%22Johns%20Hopkins%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D22" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E22" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5410,7 +6210,7 @@
         <x:v>https://www.google.com/search?q=%22University%20College%20London%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D23" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E23" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5430,7 +6230,7 @@
         <x:v>https://www.google.com/search?q=%22Imperial%20College%20London%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D24" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E24" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5450,7 +6250,7 @@
         <x:v>https://www.google.com/search?q=%22Karolinska%20Institutet%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D25" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E25" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5470,7 +6270,7 @@
         <x:v>https://www.google.com/search?q=%22ETH%20Zurich%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D26" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E26" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5484,13 +6284,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B27" s="26" t="str">
-        <x:v>"University of Oxford" "health informatics" "PhD"</x:v>
+        <x:v>"Seoul National University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C27" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20of%20Oxford%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Seoul%20National%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D27" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E27" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5504,13 +6304,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B28" s="26" t="str">
-        <x:v>"University of Cambridge" "health informatics" "PhD"</x:v>
+        <x:v>"KAIST" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C28" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20of%20Cambridge%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22KAIST%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D28" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E28" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5524,13 +6324,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B29" s="26" t="str">
-        <x:v>"University of Toronto" "health informatics" "PhD"</x:v>
+        <x:v>"Yonsei University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C29" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20of%20Toronto%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Yonsei%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D29" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E29" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5544,13 +6344,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B30" s="26" t="str">
-        <x:v>"University of Michigan" "health informatics" "PhD"</x:v>
+        <x:v>"Korea University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C30" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20of%20Michigan%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Korea%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D30" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E30" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5564,13 +6364,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B31" s="26" t="str">
-        <x:v>"Nantes Universite" "health informatics" "PhD"</x:v>
+        <x:v>"POSTECH" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C31" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22Nantes%20Universite%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22POSTECH%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D31" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E31" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5584,13 +6384,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B32" s="26" t="str">
-        <x:v>"McGill University" "health informatics" "PhD"</x:v>
+        <x:v>"Sungkyunkwan University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C32" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22McGill%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Sungkyunkwan%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D32" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E32" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5604,13 +6404,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B33" s="26" t="str">
-        <x:v>"University of British Columbia" "health informatics" "PhD"</x:v>
+        <x:v>"Hanyang University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C33" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20of%20British%20Columbia%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Hanyang%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D33" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E33" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5624,13 +6424,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B34" s="26" t="str">
-        <x:v>"Johns Hopkins University" "health informatics" "PhD"</x:v>
+        <x:v>"Ulsan National Institute of Science and Technology" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C34" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22Johns%20Hopkins%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Ulsan%20National%20Institute%20of%20Science%20and%20Technology%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D34" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E34" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5644,13 +6444,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B35" s="26" t="str">
-        <x:v>"University College London" "health informatics" "PhD"</x:v>
+        <x:v>"GIST" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C35" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22University%20College%20London%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22GIST%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D35" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E35" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5664,13 +6464,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B36" s="26" t="str">
-        <x:v>"Imperial College London" "health informatics" "PhD"</x:v>
+        <x:v>"Kyung Hee University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C36" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22Imperial%20College%20London%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Kyung%20Hee%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D36" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E36" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5684,13 +6484,13 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B37" s="26" t="str">
-        <x:v>"Karolinska Institutet" "health informatics" "PhD"</x:v>
+        <x:v>"University of Tokyo" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C37" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22Karolinska%20Institutet%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22University%20of%20Tokyo%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D37" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E37" s="26" t="str">
         <x:v>PhD advert</x:v>
@@ -5704,18 +6504,818 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="B38" s="26" t="str">
-        <x:v>"ETH Zurich" "health informatics" "PhD"</x:v>
+        <x:v>"Kyoto University" "PhD position" "medicinal chemistry"</x:v>
       </x:c>
       <x:c r="C38" s="26" t="str">
-        <x:v>https://www.google.com/search?q=%22ETH%20Zurich%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+        <x:v>https://www.google.com/search?q=%22Kyoto%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
       </x:c>
       <x:c r="D38" s="26" t="str">
-        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, university job pages, faculty lab websites</x:v>
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
       </x:c>
       <x:c r="E38" s="26" t="str">
         <x:v>PhD advert</x:v>
       </x:c>
       <x:c r="F38" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B39" s="26" t="str">
+        <x:v>"Osaka University" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C39" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Osaka%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D39" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E39" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F39" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>"Tohoku University" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Tohoku%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F40" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B41" s="26" t="str">
+        <x:v>"Nagoya University" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C41" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Nagoya%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E41" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F41" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B42" s="26" t="str">
+        <x:v>"Kyushu University" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C42" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Kyushu%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D42" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E42" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F42" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B43" s="26" t="str">
+        <x:v>"Hokkaido University" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C43" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Hokkaido%20University%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D43" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E43" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F43" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B44" s="26" t="str">
+        <x:v>"University of Tsukuba" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C44" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Tsukuba%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D44" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E44" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F44" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B45" s="26" t="str">
+        <x:v>"Institute of Science Tokyo" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C45" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Institute%20of%20Science%20Tokyo%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D45" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E45" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F45" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B46" s="26" t="str">
+        <x:v>"Okinawa Institute of Science and Technology" "PhD position" "medicinal chemistry"</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Okinawa%20Institute%20of%20Science%20and%20Technology%22%20%22PhD%20position%22%20%22medicinal%20chemistry%22</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F46" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B47" s="26" t="str">
+        <x:v>"University of Oxford" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C47" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Oxford%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F47" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="str">
+        <x:v>"University of Cambridge" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C48" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Cambridge%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F48" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B49" s="26" t="str">
+        <x:v>"University of Toronto" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C49" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Toronto%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F49" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B50" s="26" t="str">
+        <x:v>"University of Michigan" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C50" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Michigan%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F50" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B51" s="26" t="str">
+        <x:v>"Nantes Universite" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C51" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Nantes%20Universite%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F51" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B52" s="26" t="str">
+        <x:v>"McGill University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C52" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22McGill%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F52" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B53" s="26" t="str">
+        <x:v>"University of British Columbia" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C53" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20British%20Columbia%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F53" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B54" s="26" t="str">
+        <x:v>"Johns Hopkins University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C54" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Johns%20Hopkins%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F54" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B55" s="26" t="str">
+        <x:v>"University College London" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C55" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20College%20London%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F55" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B56" s="26" t="str">
+        <x:v>"Imperial College London" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C56" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Imperial%20College%20London%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D56" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F56" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B57" s="26" t="str">
+        <x:v>"Karolinska Institutet" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C57" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Karolinska%20Institutet%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D57" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F57" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B58" s="26" t="str">
+        <x:v>"ETH Zurich" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C58" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22ETH%20Zurich%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D58" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F58" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B59" s="26" t="str">
+        <x:v>"Seoul National University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C59" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Seoul%20National%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B60" s="26" t="str">
+        <x:v>"KAIST" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C60" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22KAIST%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D60" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E60" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F60" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B61" s="26" t="str">
+        <x:v>"Yonsei University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C61" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Yonsei%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D61" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E61" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F61" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B62" s="26" t="str">
+        <x:v>"Korea University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C62" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Korea%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D62" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E62" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F62" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B63" s="26" t="str">
+        <x:v>"POSTECH" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C63" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22POSTECH%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D63" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E63" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F63" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B64" s="26" t="str">
+        <x:v>"Sungkyunkwan University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C64" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Sungkyunkwan%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D64" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E64" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F64" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B65" s="26" t="str">
+        <x:v>"Hanyang University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C65" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Hanyang%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D65" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E65" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F65" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B66" s="26" t="str">
+        <x:v>"Ulsan National Institute of Science and Technology" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C66" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Ulsan%20National%20Institute%20of%20Science%20and%20Technology%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D66" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E66" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F66" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B67" s="26" t="str">
+        <x:v>"GIST" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C67" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22GIST%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D67" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E67" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F67" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B68" s="26" t="str">
+        <x:v>"Kyung Hee University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C68" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Kyung%20Hee%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D68" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E68" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F68" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B69" s="26" t="str">
+        <x:v>"University of Tokyo" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C69" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Tokyo%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D69" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E69" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F69" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B70" s="26" t="str">
+        <x:v>"Kyoto University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C70" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Kyoto%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D70" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E70" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F70" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B71" s="26" t="str">
+        <x:v>"Osaka University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C71" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Osaka%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D71" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E71" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F71" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B72" s="26" t="str">
+        <x:v>"Tohoku University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C72" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Tohoku%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D72" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E72" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F72" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B73" s="26" t="str">
+        <x:v>"Nagoya University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C73" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Nagoya%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D73" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E73" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F73" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B74" s="26" t="str">
+        <x:v>"Kyushu University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C74" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Kyushu%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D74" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E74" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F74" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B75" s="26" t="str">
+        <x:v>"Hokkaido University" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C75" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Hokkaido%20University%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D75" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E75" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F75" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B76" s="26" t="str">
+        <x:v>"University of Tsukuba" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C76" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22University%20of%20Tsukuba%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D76" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E76" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F76" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B77" s="26" t="str">
+        <x:v>"Institute of Science Tokyo" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C77" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Institute%20of%20Science%20Tokyo%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D77" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E77" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F77" s="26" t="str">
+        <x:v>Review official pages first; paste final source URL into Leads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="26" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="B78" s="26" t="str">
+        <x:v>"Okinawa Institute of Science and Technology" "health informatics" "PhD"</x:v>
+      </x:c>
+      <x:c r="C78" s="26" t="str">
+        <x:v>https://www.google.com/search?q=%22Okinawa%20Institute%20of%20Science%20and%20Technology%22%20%22health%20informatics%22%20%22PhD%22</x:v>
+      </x:c>
+      <x:c r="D78" s="26" t="str">
+        <x:v>FindAPhD, EURAXESS, Academic Positions, jobs.ac.uk, Nature Careers, JREC-IN Portal, JSPS, MEXT, Study in Korea, university job pages, faculty lab websites</x:v>
+      </x:c>
+      <x:c r="E78" s="26" t="str">
+        <x:v>PhD advert</x:v>
+      </x:c>
+      <x:c r="F78" s="26" t="str">
         <x:v>Review official pages first; paste final source URL into Leads.</x:v>
       </x:c>
     </x:row>
@@ -5726,7 +7326,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f9d89686ce941a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b6c9feba0564ab9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6598,7 +8198,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re54d760225f845bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dc8b33e6b79419e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6880,7 +8480,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0de172dd40d4b4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R079bb463d6aa4231"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7168,7 +8768,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe3b714e32e04ae7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R857dbdf312a44eeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>